<commit_message>
feat: Add 25 new scrapers (Broadridge, Carelon, Motorola Solutions, Prudential, First American, Fractal, 3M, Autodesk, Invesco, Rockwell Automation, Amadeus, Franklin Templeton, Guardian, Bloom Energy, Broadcom, Ryan, AU Small Finance, Airtel, Ashok Leyland, Experian, Freshworks, Apollo Hospitals, Biocon, GEP Worldwide, Genpact)
All 25 scrapers tested and returning jobs. Covers Workday API (16), DarwinBox (3), SmartRecruiters (2), Oracle HCM (1), SuccessFactors (1), iCIMS (1), Taleo (1). Updated registry and company-list.xlsx (331 Done, 445 Pending, 23 Broken).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -83,7 +83,7 @@
       <color rgb="009C6500"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -138,6 +138,18 @@
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0090EE90"/>
+        <bgColor rgb="0090EE90"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -151,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -245,6 +257,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1022,7 +1046,7 @@
 https://careers.ey.com/ey/search/?createNewAlert=false&amp;q=&amp;optionsFacetsDD_customfield1=&amp;optionsFacetsDD_country=IN&amp;optionsFacetsDD_city=</t>
         </is>
       </c>
-      <c r="C14" s="32" t="inlineStr">
+      <c r="C14" s="35" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -10862,9 +10886,9 @@
           <t>https://autalenthub.darwinbox.in/ms/candidatev2/main/careers/allJobs</t>
         </is>
       </c>
-      <c r="C260" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C260" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D260" s="10" t="n"/>
@@ -10902,9 +10926,9 @@
           <t>https://broadridge.wd5.myworkdayjobs.com/en-GB/Careers?Location_Country=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C261" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C261" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D261" s="10" t="n"/>
@@ -11182,9 +11206,9 @@
           <t>https://careers.smartrecruiters.com/experian</t>
         </is>
       </c>
-      <c r="C268" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C268" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D268" s="10" t="n"/>
@@ -11502,9 +11526,9 @@
           <t>https://firstam.wd1.myworkdayjobs.com/en-US/faicareers</t>
         </is>
       </c>
-      <c r="C276" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C276" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D276" s="10" t="n"/>
@@ -11542,9 +11566,9 @@
           <t>https://fractal.wd1.myworkdayjobs.com/Careers</t>
         </is>
       </c>
-      <c r="C277" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C277" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D277" s="10" t="n"/>
@@ -11662,9 +11686,9 @@
           <t>https://ryan.wd1.myworkdayjobs.com/RyanCareers?locations=9c5ef1aaea1c1050c0d408f2350b94c3&amp;locations=7cb141a2f2641001ebada432a0870000&amp;locations=313eb71192a51001a581d3bde5ea0000</t>
         </is>
       </c>
-      <c r="C280" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C280" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D280" s="10" t="n"/>
@@ -11862,9 +11886,9 @@
           <t>https://elevancehealth.wd1.myworkdayjobs.com/en-US/carelonglobal_in</t>
         </is>
       </c>
-      <c r="C285" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C285" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D285" s="10" t="n"/>
@@ -12022,9 +12046,9 @@
           <t>https://3m.wd1.myworkdayjobs.com/en-US/Search?Location_Country=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C289" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C289" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D289" s="10" t="n"/>
@@ -12262,9 +12286,9 @@
           <t>https://airtel.darwinbox.in/ms/candidatev2/main/careers/allJobs</t>
         </is>
       </c>
-      <c r="C295" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C295" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D295" s="10" t="n"/>
@@ -12382,9 +12406,9 @@
           <t>https://cgs.fa.ap2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2/jobs?location=India&amp;locationId=300000000471745&amp;locationLevel=country&amp;mode=location</t>
         </is>
       </c>
-      <c r="C298" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C298" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D298" s="10" t="n"/>
@@ -12422,7 +12446,7 @@
           <t>https://ashokleyland.darwinbox.in/ms/candidate/a61cb038c35a54/careers</t>
         </is>
       </c>
-      <c r="C299" s="32" t="inlineStr">
+      <c r="C299" s="35" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -12502,9 +12526,9 @@
           <t>https://autodesk.wd1.myworkdayjobs.com/Ext?_gl=1*1oqsxil*_gcl_au*MTgxNzc2NTUxMy4xNzcxNDk3MzE0*_ga*MTUyMTAyMzU2MC4xNzcxNDk3MzEz*_ga_NZSJ72N6RX*czE3NzE0OTczMTMkbzEkZzEkdDE3NzE0OTczMTMkajYwJGwwJGgw&amp;State_Region=701eb5584934425d930bc84b9e8b04eb&amp;State_Region=a3c37012f51642f4a7b3dafc8ac37801</t>
         </is>
       </c>
-      <c r="C301" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C301" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D301" s="10" t="n"/>
@@ -12582,9 +12606,9 @@
           <t>https://career10.successfactors.com/career?company=bioconlimi&amp;career%5fns=job%5flisting%5fsummary&amp;navBarLevel=JOB%5fSEARCH&amp;_s.crb=SzYOaazR54t4YB1PCctUttlb8GdDqA7LIeSnVs4uNqg%3d</t>
         </is>
       </c>
-      <c r="C303" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C303" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D303" s="10" t="n"/>
@@ -13625,9 +13649,9 @@
           <t>https://careers.smartrecruiters.com/Freshworks</t>
         </is>
       </c>
-      <c r="C329" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C329" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D329" s="10" t="n"/>
@@ -14025,9 +14049,9 @@
           <t>https://invesco.wd1.myworkdayjobs.com/en-GB/IVZ?locations=1804888b7f5a100128e426fb60bc0000</t>
         </is>
       </c>
-      <c r="C339" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C339" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D339" s="10" t="n"/>
@@ -14505,9 +14529,9 @@
           <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers?timeType=14bb6aa2c25e4a218b2a3faaa951e44c&amp;locationCountry=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C351" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C351" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D351" s="10" t="n"/>
@@ -14825,9 +14849,9 @@
           <t>https://prudential.wd3.myworkdayjobs.com/prudential?locationHierarchy1=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C359" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C359" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D359" s="10" t="n"/>
@@ -15224,9 +15248,9 @@
           <t>https://rockwellautomation.wd1.myworkdayjobs.com/en-US/External_Rockwell_Automation?locationCountry=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C377" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C377" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15428,9 +15452,9 @@
           <t>https://amadeus.wd502.myworkdayjobs.com/jobs?locationCountry=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C389" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C389" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15666,9 +15690,9 @@
           <t>https://franklintempleton.wd5.myworkdayjobs.com/Primary-External-1?_gl=1*q7f5r8*_ga*Njg1MzEyNTU5LjE3NzIxMDQxNjM.*_ga_15V8ZZDP8Z*czE3NzIxMDQxNjIkbzEkZzAkdDE3NzIxMDQxOTgkajI0JGwwJGgw&amp;locationCountry=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C403" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C403" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15751,9 +15775,9 @@
           <t>https://genpact.taleo.net/careersection/sgy_external_career_section/jobsearch.ftl?lang=en&amp;portal=44100025334&amp;career-search=</t>
         </is>
       </c>
-      <c r="C408" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C408" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15819,9 +15843,9 @@
           <t>https://guardianlife.wd5.myworkdayjobs.com/en-GB/Guardian-Life-Careers?locationCountry=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C412" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C412" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15921,9 +15945,9 @@
           <t>https://jobsindia-apac-gep.icims.com/jobs/search?ss=1&amp;searchRelation=keyword_all&amp;searchLocation=13228-13248-Airoli+%28W%29%2C+Navi+Mumbai</t>
         </is>
       </c>
-      <c r="C418" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C418" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16074,9 +16098,9 @@
           <t>https://bloomenergy.wd1.myworkdayjobs.com/BloomEnergyCareers?locationCountry=c4f78be1a8f14da0ab49ce1162348a5e</t>
         </is>
       </c>
-      <c r="C427" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C427" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16091,7 +16115,7 @@
           <t>https://bloomberg.avature.net/careers/SearchJobs/?1845=%5B162477%2C162478%2C162575%5D&amp;1845_format=3996&amp;listFilterMode=1&amp;jobRecordsPerPage=12&amp;</t>
         </is>
       </c>
-      <c r="C428" s="34" t="inlineStr">
+      <c r="C428" s="37" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -17210,7 +17234,7 @@
           <t>https://apollotyres.csod.com/ux/ats/careersite/1/home?c=apollotyres&amp;country=in</t>
         </is>
       </c>
-      <c r="C460" s="34" t="inlineStr">
+      <c r="C460" s="37" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -17329,9 +17353,9 @@
           <t>https://broadcom.wd1.myworkdayjobs.com/External_Career?locations=752a3c9efe39105be2259b2c18d3b6e4&amp;locations=877d747df7191002136421863fac0000&amp;locations=0dd627624e2e0176f301cad8dcd9ab0b&amp;locations=877d747df71910021363ea290d900000&amp;locations=2a204116f85f01189cd964af936b70fb</t>
         </is>
       </c>
-      <c r="C467" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C467" s="36" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -24214,7 +24238,7 @@
         </is>
       </c>
       <c r="B671" s="10" t="n"/>
-      <c r="C671" s="34" t="inlineStr">
+      <c r="C671" s="37" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -26078,9 +26102,9 @@
           <t>https://olacareers.turbohire.co/dashboardv2?orgId=e0c1eb37-eb7a-4ca4-bcc5-d59ce4ce9212&amp;type=0</t>
         </is>
       </c>
-      <c r="C722" s="32" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="C722" s="38" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="D722" s="10" t="n"/>

</xml_diff>

<commit_message>
feat: Add 25 new scrapers (Workday Inc, Otis, GE Appliances, BharatPe, JSW Group, Unacademy, Zee News, IndiaFirst Life, PharmEasy, DP World, Startek, Chubb, Essar Group, ArcelorMittal, Udacity, Groupon, Coinbase, Duolingo, Figma, InMobi, Coursera, GoDaddy, Anthropic, Truecaller, Dream11)
Tested job counts: Workday Inc 20, Otis 20, GE Appliances 14, BharatPe 4, JSW Group 3, Unacademy 7, Zee News 3, IndiaFirst Life 2, PharmEasy 10, DP World 25, Startek 25, Chubb 25, Essar Group 25, ArcelorMittal 25, Udacity 7, Groupon 4, Coinbase 11, Duolingo 2, Figma 3, InMobi 61, Coursera 12, GoDaddy 16, Anthropic 6, Truecaller 2, Dream11 26

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -11448,7 +11448,7 @@
       </c>
       <c r="C274" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D274" s="10" t="n"/>
@@ -11488,7 +11488,7 @@
       </c>
       <c r="C275" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D275" s="10" t="n"/>
@@ -13008,7 +13008,7 @@
       </c>
       <c r="C313" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D313" s="10" t="n"/>
@@ -13090,7 +13090,7 @@
       </c>
       <c r="C315" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D315" s="10" t="n"/>
@@ -13130,7 +13130,7 @@
       </c>
       <c r="C316" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D316" s="10" t="n"/>
@@ -13531,7 +13531,7 @@
       </c>
       <c r="C326" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D326" s="10" t="n"/>
@@ -13811,7 +13811,7 @@
       </c>
       <c r="C333" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D333" s="10" t="n"/>
@@ -13971,7 +13971,7 @@
       </c>
       <c r="C337" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D337" s="10" t="n"/>
@@ -14691,7 +14691,7 @@
       </c>
       <c r="C355" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D355" s="10" t="n"/>
@@ -15028,7 +15028,7 @@
       </c>
       <c r="C364" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15045,7 +15045,7 @@
       </c>
       <c r="C365" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15301,7 +15301,7 @@
       </c>
       <c r="C380" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15352,7 +15352,7 @@
       </c>
       <c r="C383" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15369,7 +15369,7 @@
       </c>
       <c r="C384" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15726,7 +15726,7 @@
       </c>
       <c r="C405" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16396,7 +16396,7 @@
       </c>
       <c r="C439" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D439" s="10" t="n"/>
@@ -16876,7 +16876,7 @@
       </c>
       <c r="C451" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D451" s="10" t="n"/>
@@ -17036,7 +17036,7 @@
       </c>
       <c r="C455" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D455" s="10" t="n"/>
@@ -17253,7 +17253,7 @@
       </c>
       <c r="C461" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17460,7 +17460,7 @@
       </c>
       <c r="C473" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17477,7 +17477,7 @@
       </c>
       <c r="C474" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17630,7 +17630,7 @@
       </c>
       <c r="C483" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17715,7 +17715,7 @@
       </c>
       <c r="C488" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17766,7 +17766,7 @@
       </c>
       <c r="C491" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17868,7 +17868,7 @@
       </c>
       <c r="C497" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add 25 new scrapers (Batch 3) - Greenhouse, Lever, Workday APIs + CLAUDE.md rules
Greenhouse API (17): Airbnb, Agoda, Capco, Groww, Postman, Druva, Databricks, Okta, Zscaler, Stripe, Rubrik, MongoDB, Toast, SumoLogic, Elastic, Twilio, Datadog
Lever API (3): Spotify, Binance, CRED
Workday API (5): Stryker, Amgen, Kenvue, Athenahealth, Bristol-Myers Squibb

All scrapers tested with multipage verification. Added CLAUDE.md with comprehensive scraper development rules.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1242"/>
+  <dimension ref="A1:Z1256"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="25.13" customWidth="1" style="26" min="1" max="1"/>
@@ -11248,7 +11248,7 @@
       </c>
       <c r="C269" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D269" s="10" t="n"/>
@@ -12248,7 +12248,7 @@
       </c>
       <c r="C294" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D294" s="10" t="n"/>
@@ -12328,7 +12328,7 @@
       </c>
       <c r="C296" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D296" s="10" t="n"/>
@@ -12768,7 +12768,7 @@
       </c>
       <c r="C307" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D307" s="10" t="n"/>
@@ -13170,7 +13170,7 @@
       </c>
       <c r="C317" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D317" s="10" t="n"/>
@@ -14171,7 +14171,7 @@
       </c>
       <c r="C342" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D342" s="10" t="n"/>
@@ -15539,7 +15539,7 @@
       </c>
       <c r="C394" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15573,7 +15573,7 @@
       </c>
       <c r="C396" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C425" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16676,7 +16676,7 @@
       </c>
       <c r="C446" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D446" s="10" t="n"/>
@@ -17287,7 +17287,7 @@
       </c>
       <c r="C463" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -41125,6 +41125,244 @@
       <c r="X1242" s="10" t="n"/>
       <c r="Y1242" s="10" t="n"/>
       <c r="Z1242" s="10" t="n"/>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/groww</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>Postman</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/postman</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>Druva</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/druva</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/databricks</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>Okta</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/okta</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>Zscaler</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/zscaler</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/stripe</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>Rubrik</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/rubrik</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/mongodb</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/toast</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>Sumo Logic</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/sumologic</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>Elastic</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/elastic</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>Twilio</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/twilio</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>Datadog</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/datadog</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
feat: Add 25 new scrapers (Batch 4) - Greenhouse and Lever APIs
Greenhouse API (24): Five9, Tekion, Celonis, CloudSEK, Zuora, SolarWinds, Aviatrix, Fivetran, OneTrust, Commvault, ZoomInfo, Moveworks, Vonage, Cision, Flexport, Oportun, Cockroach Labs, GitLab, DeepMind, Fastly, Karat, AppDirect, LogicMonitor, SingleStore
Lever API (1): Clari

All scrapers tested with multipage verification (single API call, no pagination needed).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1256"/>
+  <dimension ref="A1:Z1281"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="25.13" customWidth="1" style="26" min="1" max="1"/>
@@ -41127,238 +41127,538 @@
       <c r="Z1242" s="10" t="n"/>
     </row>
     <row r="1243">
-      <c r="A1243" t="inlineStr">
+      <c r="A1243" s="0" t="inlineStr">
         <is>
           <t>Groww</t>
         </is>
       </c>
-      <c r="B1243" t="inlineStr">
+      <c r="B1243" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/groww</t>
         </is>
       </c>
-      <c r="C1243" t="inlineStr">
+      <c r="C1243" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1244">
-      <c r="A1244" t="inlineStr">
+      <c r="A1244" s="0" t="inlineStr">
         <is>
           <t>Postman</t>
         </is>
       </c>
-      <c r="B1244" t="inlineStr">
+      <c r="B1244" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/postman</t>
         </is>
       </c>
-      <c r="C1244" t="inlineStr">
+      <c r="C1244" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1245">
-      <c r="A1245" t="inlineStr">
+      <c r="A1245" s="0" t="inlineStr">
         <is>
           <t>Druva</t>
         </is>
       </c>
-      <c r="B1245" t="inlineStr">
+      <c r="B1245" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/druva</t>
         </is>
       </c>
-      <c r="C1245" t="inlineStr">
+      <c r="C1245" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1246">
-      <c r="A1246" t="inlineStr">
+      <c r="A1246" s="0" t="inlineStr">
         <is>
           <t>Databricks</t>
         </is>
       </c>
-      <c r="B1246" t="inlineStr">
+      <c r="B1246" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/databricks</t>
         </is>
       </c>
-      <c r="C1246" t="inlineStr">
+      <c r="C1246" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1247">
-      <c r="A1247" t="inlineStr">
+      <c r="A1247" s="0" t="inlineStr">
         <is>
           <t>Okta</t>
         </is>
       </c>
-      <c r="B1247" t="inlineStr">
+      <c r="B1247" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/okta</t>
         </is>
       </c>
-      <c r="C1247" t="inlineStr">
+      <c r="C1247" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1248">
-      <c r="A1248" t="inlineStr">
+      <c r="A1248" s="0" t="inlineStr">
         <is>
           <t>Zscaler</t>
         </is>
       </c>
-      <c r="B1248" t="inlineStr">
+      <c r="B1248" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/zscaler</t>
         </is>
       </c>
-      <c r="C1248" t="inlineStr">
+      <c r="C1248" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1249">
-      <c r="A1249" t="inlineStr">
+      <c r="A1249" s="0" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="B1249" t="inlineStr">
+      <c r="B1249" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/stripe</t>
         </is>
       </c>
-      <c r="C1249" t="inlineStr">
+      <c r="C1249" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1250">
-      <c r="A1250" t="inlineStr">
+      <c r="A1250" s="0" t="inlineStr">
         <is>
           <t>Rubrik</t>
         </is>
       </c>
-      <c r="B1250" t="inlineStr">
+      <c r="B1250" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/rubrik</t>
         </is>
       </c>
-      <c r="C1250" t="inlineStr">
+      <c r="C1250" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1251">
-      <c r="A1251" t="inlineStr">
+      <c r="A1251" s="0" t="inlineStr">
         <is>
           <t>MongoDB</t>
         </is>
       </c>
-      <c r="B1251" t="inlineStr">
+      <c r="B1251" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/mongodb</t>
         </is>
       </c>
-      <c r="C1251" t="inlineStr">
+      <c r="C1251" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1252">
-      <c r="A1252" t="inlineStr">
+      <c r="A1252" s="0" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
-      <c r="B1252" t="inlineStr">
+      <c r="B1252" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/toast</t>
         </is>
       </c>
-      <c r="C1252" t="inlineStr">
+      <c r="C1252" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1253">
-      <c r="A1253" t="inlineStr">
+      <c r="A1253" s="0" t="inlineStr">
         <is>
           <t>Sumo Logic</t>
         </is>
       </c>
-      <c r="B1253" t="inlineStr">
+      <c r="B1253" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/sumologic</t>
         </is>
       </c>
-      <c r="C1253" t="inlineStr">
+      <c r="C1253" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1254">
-      <c r="A1254" t="inlineStr">
+      <c r="A1254" s="0" t="inlineStr">
         <is>
           <t>Elastic</t>
         </is>
       </c>
-      <c r="B1254" t="inlineStr">
+      <c r="B1254" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/elastic</t>
         </is>
       </c>
-      <c r="C1254" t="inlineStr">
+      <c r="C1254" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1255">
-      <c r="A1255" t="inlineStr">
+      <c r="A1255" s="0" t="inlineStr">
         <is>
           <t>Twilio</t>
         </is>
       </c>
-      <c r="B1255" t="inlineStr">
+      <c r="B1255" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/twilio</t>
         </is>
       </c>
-      <c r="C1255" t="inlineStr">
+      <c r="C1255" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1256">
-      <c r="A1256" t="inlineStr">
+      <c r="A1256" s="0" t="inlineStr">
         <is>
           <t>Datadog</t>
         </is>
       </c>
-      <c r="B1256" t="inlineStr">
+      <c r="B1256" s="0" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/datadog</t>
         </is>
       </c>
-      <c r="C1256" t="inlineStr">
+      <c r="C1256" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>Five9</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>Tekion</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>Celonis</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>CloudSEK</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>Zuora</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>SolarWinds</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>Aviatrix</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>Fivetran</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>OneTrust</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>Commvault</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>ZoomInfo</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>Moveworks</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>Vonage</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>Cision</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>Flexport</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>Oportun</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>Cockroach Labs</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>GitLab</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>DeepMind</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>Fastly</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>Karat</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>AppDirect</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>LogicMonitor</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>SingleStore</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>Clari</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
feat: Add 25 new scrapers (Batch 5) - Greenhouse, Workday APIs
Greenhouse API (21): Netskope, Fictiv, Zenoti, DevRev, HackerRank, SmartBear, BitGo, New Relic, Bloomreach, Turing, Britive, Zocdoc, Narvar, Workato, Project44, Yugabyte, Thoughtworks, Starburst, Backblaze, Catchpoint, Sendbird
Workday API (4): Mastercard, Medtronic, PayPal, Zoom

All scrapers tested with multipage verification. Workday pagination uses page counter for searchText scrapers.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1281"/>
+  <dimension ref="A1:Z1303"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="25.13" customWidth="1" style="26" min="1" max="1"/>
@@ -14411,7 +14411,7 @@
       </c>
       <c r="C348" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D348" s="10" t="n"/>
@@ -14731,7 +14731,7 @@
       </c>
       <c r="C356" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D356" s="10" t="n"/>
@@ -16356,7 +16356,7 @@
       </c>
       <c r="C438" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D438" s="10" t="n"/>
@@ -41365,300 +41365,564 @@
       </c>
     </row>
     <row r="1257">
-      <c r="A1257" t="inlineStr">
+      <c r="A1257" s="0" t="inlineStr">
         <is>
           <t>Five9</t>
         </is>
       </c>
-      <c r="C1257" t="inlineStr">
+      <c r="C1257" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1258">
-      <c r="A1258" t="inlineStr">
+      <c r="A1258" s="0" t="inlineStr">
         <is>
           <t>Tekion</t>
         </is>
       </c>
-      <c r="C1258" t="inlineStr">
+      <c r="C1258" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1259">
-      <c r="A1259" t="inlineStr">
+      <c r="A1259" s="0" t="inlineStr">
         <is>
           <t>Celonis</t>
         </is>
       </c>
-      <c r="C1259" t="inlineStr">
+      <c r="C1259" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1260">
-      <c r="A1260" t="inlineStr">
+      <c r="A1260" s="0" t="inlineStr">
         <is>
           <t>CloudSEK</t>
         </is>
       </c>
-      <c r="C1260" t="inlineStr">
+      <c r="C1260" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1261">
-      <c r="A1261" t="inlineStr">
+      <c r="A1261" s="0" t="inlineStr">
         <is>
           <t>Zuora</t>
         </is>
       </c>
-      <c r="C1261" t="inlineStr">
+      <c r="C1261" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1262">
-      <c r="A1262" t="inlineStr">
+      <c r="A1262" s="0" t="inlineStr">
         <is>
           <t>SolarWinds</t>
         </is>
       </c>
-      <c r="C1262" t="inlineStr">
+      <c r="C1262" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1263">
-      <c r="A1263" t="inlineStr">
+      <c r="A1263" s="0" t="inlineStr">
         <is>
           <t>Aviatrix</t>
         </is>
       </c>
-      <c r="C1263" t="inlineStr">
+      <c r="C1263" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1264">
-      <c r="A1264" t="inlineStr">
+      <c r="A1264" s="0" t="inlineStr">
         <is>
           <t>Fivetran</t>
         </is>
       </c>
-      <c r="C1264" t="inlineStr">
+      <c r="C1264" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1265">
-      <c r="A1265" t="inlineStr">
+      <c r="A1265" s="0" t="inlineStr">
         <is>
           <t>OneTrust</t>
         </is>
       </c>
-      <c r="C1265" t="inlineStr">
+      <c r="C1265" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1266">
-      <c r="A1266" t="inlineStr">
+      <c r="A1266" s="0" t="inlineStr">
         <is>
           <t>Commvault</t>
         </is>
       </c>
-      <c r="C1266" t="inlineStr">
+      <c r="C1266" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1267">
-      <c r="A1267" t="inlineStr">
+      <c r="A1267" s="0" t="inlineStr">
         <is>
           <t>ZoomInfo</t>
         </is>
       </c>
-      <c r="C1267" t="inlineStr">
+      <c r="C1267" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1268">
-      <c r="A1268" t="inlineStr">
+      <c r="A1268" s="0" t="inlineStr">
         <is>
           <t>Moveworks</t>
         </is>
       </c>
-      <c r="C1268" t="inlineStr">
+      <c r="C1268" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1269">
-      <c r="A1269" t="inlineStr">
+      <c r="A1269" s="0" t="inlineStr">
         <is>
           <t>Vonage</t>
         </is>
       </c>
-      <c r="C1269" t="inlineStr">
+      <c r="C1269" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1270">
-      <c r="A1270" t="inlineStr">
+      <c r="A1270" s="0" t="inlineStr">
         <is>
           <t>Cision</t>
         </is>
       </c>
-      <c r="C1270" t="inlineStr">
+      <c r="C1270" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1271">
-      <c r="A1271" t="inlineStr">
+      <c r="A1271" s="0" t="inlineStr">
         <is>
           <t>Flexport</t>
         </is>
       </c>
-      <c r="C1271" t="inlineStr">
+      <c r="C1271" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1272">
-      <c r="A1272" t="inlineStr">
+      <c r="A1272" s="0" t="inlineStr">
         <is>
           <t>Oportun</t>
         </is>
       </c>
-      <c r="C1272" t="inlineStr">
+      <c r="C1272" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1273">
-      <c r="A1273" t="inlineStr">
+      <c r="A1273" s="0" t="inlineStr">
         <is>
           <t>Cockroach Labs</t>
         </is>
       </c>
-      <c r="C1273" t="inlineStr">
+      <c r="C1273" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1274">
-      <c r="A1274" t="inlineStr">
+      <c r="A1274" s="0" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="C1274" t="inlineStr">
+      <c r="C1274" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1275">
-      <c r="A1275" t="inlineStr">
+      <c r="A1275" s="0" t="inlineStr">
         <is>
           <t>DeepMind</t>
         </is>
       </c>
-      <c r="C1275" t="inlineStr">
+      <c r="C1275" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1276">
-      <c r="A1276" t="inlineStr">
+      <c r="A1276" s="0" t="inlineStr">
         <is>
           <t>Fastly</t>
         </is>
       </c>
-      <c r="C1276" t="inlineStr">
+      <c r="C1276" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1277">
-      <c r="A1277" t="inlineStr">
+      <c r="A1277" s="0" t="inlineStr">
         <is>
           <t>Karat</t>
         </is>
       </c>
-      <c r="C1277" t="inlineStr">
+      <c r="C1277" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1278">
-      <c r="A1278" t="inlineStr">
+      <c r="A1278" s="0" t="inlineStr">
         <is>
           <t>AppDirect</t>
         </is>
       </c>
-      <c r="C1278" t="inlineStr">
+      <c r="C1278" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1279">
-      <c r="A1279" t="inlineStr">
+      <c r="A1279" s="0" t="inlineStr">
         <is>
           <t>LogicMonitor</t>
         </is>
       </c>
-      <c r="C1279" t="inlineStr">
+      <c r="C1279" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1280">
-      <c r="A1280" t="inlineStr">
+      <c r="A1280" s="0" t="inlineStr">
         <is>
           <t>SingleStore</t>
         </is>
       </c>
-      <c r="C1280" t="inlineStr">
+      <c r="C1280" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1281">
-      <c r="A1281" t="inlineStr">
+      <c r="A1281" s="0" t="inlineStr">
         <is>
           <t>Clari</t>
         </is>
       </c>
-      <c r="C1281" t="inlineStr">
+      <c r="C1281" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>Netskope</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>Fictiv</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>Zenoti</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>DevRev</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>HackerRank</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>SmartBear</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>BitGo</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>New Relic</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>Bloomreach</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>Britive</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>Zocdoc</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>Narvar</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>Workato</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>Project44</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>Yugabyte</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>Thoughtworks</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>Starburst</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>Backblaze</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>Catchpoint</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>Sendbird</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>Medtronic</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
feat: Add 23 new scrapers (Batch 6) - Greenhouse and Lever APIs
HighRadius(33), Anaplan(30), Kaseya(24), Quince(19), ChargePoint(16),
Appian(13), Plume(11), 6sense(11), Abnormal Security(9), Dialpad(8),
Suki(8), FalconX(7), Everbridge(7), Ivalua(6), Greenlight(6),
Mindbody(4), JustAnswer(4), Cresta(3), Blueshift(2), Biofourmis(1),
MinIO(1), KnowBe4(1), Coupang(40) - 264 total India jobs

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -41665,264 +41665,264 @@
       </c>
     </row>
     <row r="1282">
-      <c r="A1282" t="inlineStr">
+      <c r="A1282" s="0" t="inlineStr">
         <is>
           <t>Netskope</t>
         </is>
       </c>
-      <c r="C1282" t="inlineStr">
+      <c r="C1282" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1283">
-      <c r="A1283" t="inlineStr">
+      <c r="A1283" s="0" t="inlineStr">
         <is>
           <t>Fictiv</t>
         </is>
       </c>
-      <c r="C1283" t="inlineStr">
+      <c r="C1283" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1284">
-      <c r="A1284" t="inlineStr">
+      <c r="A1284" s="0" t="inlineStr">
         <is>
           <t>Zenoti</t>
         </is>
       </c>
-      <c r="C1284" t="inlineStr">
+      <c r="C1284" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1285">
-      <c r="A1285" t="inlineStr">
+      <c r="A1285" s="0" t="inlineStr">
         <is>
           <t>DevRev</t>
         </is>
       </c>
-      <c r="C1285" t="inlineStr">
+      <c r="C1285" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1286">
-      <c r="A1286" t="inlineStr">
+      <c r="A1286" s="0" t="inlineStr">
         <is>
           <t>HackerRank</t>
         </is>
       </c>
-      <c r="C1286" t="inlineStr">
+      <c r="C1286" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1287">
-      <c r="A1287" t="inlineStr">
+      <c r="A1287" s="0" t="inlineStr">
         <is>
           <t>SmartBear</t>
         </is>
       </c>
-      <c r="C1287" t="inlineStr">
+      <c r="C1287" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1288">
-      <c r="A1288" t="inlineStr">
+      <c r="A1288" s="0" t="inlineStr">
         <is>
           <t>BitGo</t>
         </is>
       </c>
-      <c r="C1288" t="inlineStr">
+      <c r="C1288" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1289">
-      <c r="A1289" t="inlineStr">
+      <c r="A1289" s="0" t="inlineStr">
         <is>
           <t>New Relic</t>
         </is>
       </c>
-      <c r="C1289" t="inlineStr">
+      <c r="C1289" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1290">
-      <c r="A1290" t="inlineStr">
+      <c r="A1290" s="0" t="inlineStr">
         <is>
           <t>Bloomreach</t>
         </is>
       </c>
-      <c r="C1290" t="inlineStr">
+      <c r="C1290" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1291">
-      <c r="A1291" t="inlineStr">
+      <c r="A1291" s="0" t="inlineStr">
         <is>
           <t>Turing</t>
         </is>
       </c>
-      <c r="C1291" t="inlineStr">
+      <c r="C1291" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1292">
-      <c r="A1292" t="inlineStr">
+      <c r="A1292" s="0" t="inlineStr">
         <is>
           <t>Britive</t>
         </is>
       </c>
-      <c r="C1292" t="inlineStr">
+      <c r="C1292" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1293">
-      <c r="A1293" t="inlineStr">
+      <c r="A1293" s="0" t="inlineStr">
         <is>
           <t>Zocdoc</t>
         </is>
       </c>
-      <c r="C1293" t="inlineStr">
+      <c r="C1293" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1294">
-      <c r="A1294" t="inlineStr">
+      <c r="A1294" s="0" t="inlineStr">
         <is>
           <t>Narvar</t>
         </is>
       </c>
-      <c r="C1294" t="inlineStr">
+      <c r="C1294" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1295">
-      <c r="A1295" t="inlineStr">
+      <c r="A1295" s="0" t="inlineStr">
         <is>
           <t>Workato</t>
         </is>
       </c>
-      <c r="C1295" t="inlineStr">
+      <c r="C1295" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1296">
-      <c r="A1296" t="inlineStr">
+      <c r="A1296" s="0" t="inlineStr">
         <is>
           <t>Project44</t>
         </is>
       </c>
-      <c r="C1296" t="inlineStr">
+      <c r="C1296" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1297">
-      <c r="A1297" t="inlineStr">
+      <c r="A1297" s="0" t="inlineStr">
         <is>
           <t>Yugabyte</t>
         </is>
       </c>
-      <c r="C1297" t="inlineStr">
+      <c r="C1297" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1298">
-      <c r="A1298" t="inlineStr">
+      <c r="A1298" s="0" t="inlineStr">
         <is>
           <t>Thoughtworks</t>
         </is>
       </c>
-      <c r="C1298" t="inlineStr">
+      <c r="C1298" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1299">
-      <c r="A1299" t="inlineStr">
+      <c r="A1299" s="0" t="inlineStr">
         <is>
           <t>Starburst</t>
         </is>
       </c>
-      <c r="C1299" t="inlineStr">
+      <c r="C1299" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1300">
-      <c r="A1300" t="inlineStr">
+      <c r="A1300" s="0" t="inlineStr">
         <is>
           <t>Backblaze</t>
         </is>
       </c>
-      <c r="C1300" t="inlineStr">
+      <c r="C1300" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1301">
-      <c r="A1301" t="inlineStr">
+      <c r="A1301" s="0" t="inlineStr">
         <is>
           <t>Catchpoint</t>
         </is>
       </c>
-      <c r="C1301" t="inlineStr">
+      <c r="C1301" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1302">
-      <c r="A1302" t="inlineStr">
+      <c r="A1302" s="0" t="inlineStr">
         <is>
           <t>Sendbird</t>
         </is>
       </c>
-      <c r="C1302" t="inlineStr">
+      <c r="C1302" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1303">
-      <c r="A1303" t="inlineStr">
+      <c r="A1303" s="0" t="inlineStr">
         <is>
           <t>Medtronic</t>
         </is>
       </c>
-      <c r="C1303" t="inlineStr">
+      <c r="C1303" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
feat: Add 23 new scrapers (Batch 7) - Workday, Greenhouse, and Lever APIs
16 Workday scrapers (Collins Aerospace, GE Vernova, Capital One, Maersk,
Expedia Group, Chevron, eBay, Dow, HPE, Allstate, Aptiv, Caterpillar,
Blue Yonder, Gartner, BlackRock, Becton Dickinson), 6 Greenhouse scrapers
(WPP, Encora, FlixBus, Instabase, Axon, Udemy), and 1 Lever scraper
(LinkedIn). Total: 364 India jobs across 23 companies.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -10968,7 +10968,7 @@
       </c>
       <c r="C262" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D262" s="10" t="n"/>
@@ -11008,7 +11008,7 @@
       </c>
       <c r="C263" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D263" s="10" t="n"/>
@@ -11128,7 +11128,7 @@
       </c>
       <c r="C266" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D266" s="10" t="n"/>
@@ -12568,7 +12568,7 @@
       </c>
       <c r="C302" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D302" s="10" t="n"/>
@@ -12648,7 +12648,7 @@
       </c>
       <c r="C304" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D304" s="10" t="n"/>
@@ -12848,7 +12848,7 @@
       </c>
       <c r="C309" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D309" s="10" t="n"/>
@@ -13290,7 +13290,7 @@
       </c>
       <c r="C320" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D320" s="10" t="n"/>
@@ -13571,7 +13571,7 @@
       </c>
       <c r="C327" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D327" s="10" t="n"/>
@@ -13611,7 +13611,7 @@
       </c>
       <c r="C328" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D328" s="10" t="n"/>
@@ -13731,7 +13731,7 @@
       </c>
       <c r="C331" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D331" s="10" t="n"/>
@@ -14251,7 +14251,7 @@
       </c>
       <c r="C344" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D344" s="10" t="n"/>
@@ -15011,7 +15011,7 @@
       </c>
       <c r="C363" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15403,7 +15403,7 @@
       </c>
       <c r="C386" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15522,7 +15522,7 @@
       </c>
       <c r="C393" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15624,7 +15624,7 @@
       </c>
       <c r="C399" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15641,7 +15641,7 @@
       </c>
       <c r="C400" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15743,7 +15743,7 @@
       </c>
       <c r="C406" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15828,7 +15828,7 @@
       </c>
       <c r="C411" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16236,7 +16236,7 @@
       </c>
       <c r="C435" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D435" s="10" t="n"/>
@@ -23814,7 +23814,7 @@
       <c r="B659" s="10" t="n"/>
       <c r="C659" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D659" s="10" t="n"/>

</xml_diff>

<commit_message>
feat: Add 5 new scrapers and update 4 Oracle HCM scrapers (Batch 8) - Workday, Greenhouse, SmartRecruiters, Oracle HCM APIs
New scrapers: Leidos (Workday), GE HealthCare (Workday), KKR (Greenhouse), Accor (SmartRecruiters), H&M (SmartRecruiters)
Updated: DP World, Startek, Chubb, Essar Group (Oracle HCM with India location facets)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -11408,7 +11408,7 @@
       </c>
       <c r="C273" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D273" s="10" t="n"/>
@@ -12928,7 +12928,7 @@
       </c>
       <c r="C311" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D311" s="10" t="n"/>
@@ -13370,7 +13370,7 @@
       </c>
       <c r="C322" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D322" s="10" t="n"/>
@@ -13771,7 +13771,7 @@
       </c>
       <c r="C332" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D332" s="10" t="n"/>
@@ -14211,7 +14211,7 @@
       </c>
       <c r="C343" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D343" s="10" t="n"/>
@@ -15420,7 +15420,7 @@
       </c>
       <c r="C387" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15862,7 +15862,7 @@
       </c>
       <c r="C413" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="C475" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add 6 new Ashby API scrapers (Batch 15) - Notion, OpenAI, Snowflake, Deel, Confluent, Anyscale
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1303"/>
+  <dimension ref="A1:Z1306"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="25.13" customWidth="1" style="26" min="1" max="1"/>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="C354" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D354" s="10" t="n"/>
@@ -15062,7 +15062,7 @@
       </c>
       <c r="C366" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15131,7 +15131,7 @@
       </c>
       <c r="C370" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -41923,6 +41923,57 @@
         </is>
       </c>
       <c r="C1303" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>Deel</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>Confluent</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>Anyscale</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
feat: Add 15 new scrapers (Batch 16) - DarwinBox and MakeMyTrip custom API
- 12 DarwinBox v2 Selenium scrapers: Emcure, Rapido, MG Motors, Supreme Industries,
  Lenskart, CARS24, NoBroker, Pine Labs, MobiKwik, ShareChat, Urban Company, Gupshup
- 2 DarwinBox v1 Selenium scrapers: Epson, Bonn Group
- 1 Custom JSON API scraper: MakeMyTrip (45 India jobs)
- Updated registry.py (555 SCRAPER_MAP entries, 472 ALL_COMPANY_CHOICES)
- Updated company-list.xlsx (Done: 480, Pending: 368, Broken: 23)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1306"/>
+  <dimension ref="A1:Z1314"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="25.13" customWidth="1" style="26" min="1" max="1"/>
@@ -14371,7 +14371,7 @@
       </c>
       <c r="C347" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D347" s="10" t="n"/>
@@ -15896,7 +15896,7 @@
       </c>
       <c r="C415" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16436,7 +16436,7 @@
       </c>
       <c r="C440" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D440" s="10" t="n"/>
@@ -17321,7 +17321,7 @@
       </c>
       <c r="C465" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -17528,7 +17528,7 @@
       </c>
       <c r="C477" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -22718,7 +22718,7 @@
       </c>
       <c r="C630" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D630" s="10" t="n"/>
@@ -26628,7 +26628,7 @@
       </c>
       <c r="C736" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D736" s="10" t="n"/>
@@ -41929,51 +41929,147 @@
       </c>
     </row>
     <row r="1304">
-      <c r="A1304" t="inlineStr">
+      <c r="A1304" s="0" t="inlineStr">
         <is>
           <t>Deel</t>
         </is>
       </c>
-      <c r="B1304" t="inlineStr">
+      <c r="B1304" s="0" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C1304" t="inlineStr">
+      <c r="C1304" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1305">
-      <c r="A1305" t="inlineStr">
+      <c r="A1305" s="0" t="inlineStr">
         <is>
           <t>Confluent</t>
         </is>
       </c>
-      <c r="B1305" t="inlineStr">
+      <c r="B1305" s="0" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C1305" t="inlineStr">
+      <c r="C1305" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="1306">
-      <c r="A1306" t="inlineStr">
+      <c r="A1306" s="0" t="inlineStr">
         <is>
           <t>Anyscale</t>
         </is>
       </c>
-      <c r="B1306" t="inlineStr">
+      <c r="B1306" s="0" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C1306" t="inlineStr">
+      <c r="C1306" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>Lenskart</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>CARS24</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>NoBroker</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>Pine Labs</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>MobiKwik</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>ShareChat</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>Urban Company</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>Gupshup</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
fix: Update colour key counts in company-list.xlsx (Done=499, Pending=368, Broken=4)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -589,7 +589,7 @@
       <c r="A2" s="3" t="n"/>
       <c r="B2" s="27" t="inlineStr">
         <is>
-          <t>Done (308)</t>
+          <t>Done (499)</t>
         </is>
       </c>
       <c r="C2" s="10" t="n"/>
@@ -621,7 +621,7 @@
       <c r="A3" s="4" t="n"/>
       <c r="B3" s="28" t="inlineStr">
         <is>
-          <t>Pending (468)</t>
+          <t>Pending (368)</t>
         </is>
       </c>
       <c r="C3" s="10" t="n"/>
@@ -653,7 +653,7 @@
       <c r="A4" s="5" t="n"/>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>Broken (23)</t>
+          <t>Broken (4)</t>
         </is>
       </c>
       <c r="C4" s="10" t="n"/>

</xml_diff>

<commit_message>
feat: Add 22 new scrapers (Batch 18) for ADP, Aon, Atlassian, BNY, CBRE, Cloudflare, EA, EPAM and more
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -169,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -357,6 +357,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -676,7 +682,7 @@
       <c r="A2" s="3" t="n"/>
       <c r="B2" s="27" t="inlineStr">
         <is>
-          <t>Done (523)</t>
+          <t>Done (544)</t>
         </is>
       </c>
       <c r="C2" s="10" t="n"/>
@@ -708,7 +714,7 @@
       <c r="A3" s="4" t="n"/>
       <c r="B3" s="28" t="inlineStr">
         <is>
-          <t>Pending (344)</t>
+          <t>Pending (322)</t>
         </is>
       </c>
       <c r="C3" s="10" t="n"/>
@@ -740,7 +746,7 @@
       <c r="A4" s="5" t="n"/>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>Broken (4)</t>
+          <t>Broken (5)</t>
         </is>
       </c>
       <c r="C4" s="10" t="n"/>
@@ -11883,19 +11889,19 @@
       <c r="Z282" s="10" t="n"/>
     </row>
     <row r="283">
-      <c r="A283" s="52" t="inlineStr">
+      <c r="A283" s="43" t="inlineStr">
         <is>
           <t>MSC Technology</t>
         </is>
       </c>
-      <c r="B283" s="53" t="inlineStr">
+      <c r="B283" s="44" t="inlineStr">
         <is>
           <t>https://www.msc-technology.com/current-opening-india</t>
         </is>
       </c>
-      <c r="C283" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C283" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D283" s="10" t="n"/>
@@ -12003,19 +12009,19 @@
       <c r="Z285" s="10" t="n"/>
     </row>
     <row r="286">
-      <c r="A286" s="52" t="inlineStr">
+      <c r="A286" s="43" t="inlineStr">
         <is>
           <t>HashedIn</t>
         </is>
       </c>
-      <c r="B286" s="53" t="inlineStr">
+      <c r="B286" s="44" t="inlineStr">
         <is>
           <t>https://hashedin.com/careers</t>
         </is>
       </c>
-      <c r="C286" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C286" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D286" s="10" t="n"/>
@@ -12083,19 +12089,19 @@
       <c r="Z287" s="10" t="n"/>
     </row>
     <row r="288">
-      <c r="A288" s="52" t="inlineStr">
+      <c r="A288" s="43" t="inlineStr">
         <is>
           <t>HTC Global</t>
         </is>
       </c>
-      <c r="B288" s="53" t="inlineStr">
+      <c r="B288" s="44" t="inlineStr">
         <is>
           <t>https://www.htcinc.com/career-job-listing/</t>
         </is>
       </c>
-      <c r="C288" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C288" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D288" s="10" t="n"/>
@@ -12163,19 +12169,19 @@
       <c r="Z289" s="10" t="n"/>
     </row>
     <row r="290">
-      <c r="A290" s="56" t="inlineStr">
+      <c r="A290" s="54" t="inlineStr">
         <is>
           <t>Acko</t>
         </is>
       </c>
-      <c r="B290" s="57" t="inlineStr">
+      <c r="B290" s="55" t="inlineStr">
         <is>
           <t>https://www.acko.com/careers/jobs/</t>
         </is>
       </c>
-      <c r="C290" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C290" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D290" s="10" t="n"/>
@@ -12243,19 +12249,19 @@
       <c r="Z291" s="10" t="n"/>
     </row>
     <row r="292">
-      <c r="A292" s="56" t="inlineStr">
+      <c r="A292" s="54" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="B292" s="57" t="inlineStr">
+      <c r="B292" s="55" t="inlineStr">
         <is>
           <t>https://jobs.adp.com/en/jobs/?orderby=0&amp;pagesize=20&amp;page=1&amp;mylocation=India&amp;radius=100&amp;rType=0</t>
         </is>
       </c>
-      <c r="C292" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C292" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D292" s="10" t="n"/>
@@ -12443,19 +12449,19 @@
       <c r="Z296" s="10" t="n"/>
     </row>
     <row r="297">
-      <c r="A297" s="52" t="inlineStr">
+      <c r="A297" s="43" t="inlineStr">
         <is>
           <t>Aon</t>
         </is>
       </c>
-      <c r="B297" s="53" t="inlineStr">
+      <c r="B297" s="44" t="inlineStr">
         <is>
           <t>https://jobs.aon.com/jobs?locations=Bangalore,Karnataka,India%7CBengaluru,Karnataka,India%7CGreater%20Noida,Uttar%20Pradesh,India%7CGurgaon,Haryana,India%7CGurugram,Haryana,India%7CMumbai,Maharashtra,India%7CNOIDA,Uttar%20Pradesh,India&amp;page=1</t>
         </is>
       </c>
-      <c r="C297" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C297" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D297" s="10" t="n"/>
@@ -12563,19 +12569,19 @@
       <c r="Z299" s="10" t="n"/>
     </row>
     <row r="300">
-      <c r="A300" s="56" t="inlineStr">
+      <c r="A300" s="54" t="inlineStr">
         <is>
           <t>Atlassian</t>
         </is>
       </c>
-      <c r="B300" s="53" t="inlineStr">
+      <c r="B300" s="44" t="inlineStr">
         <is>
           <t>https://www.atlassian.com/company/careers/all-jobs?team=&amp;location=India&amp;search=</t>
         </is>
       </c>
-      <c r="C300" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C300" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D300" s="10" t="n"/>
@@ -12763,19 +12769,19 @@
       <c r="Z304" s="10" t="n"/>
     </row>
     <row r="305">
-      <c r="A305" s="52" t="inlineStr">
+      <c r="A305" s="43" t="inlineStr">
         <is>
           <t>Blue Star</t>
         </is>
       </c>
-      <c r="B305" s="53" t="inlineStr">
+      <c r="B305" s="44" t="inlineStr">
         <is>
           <t>https://bluestar.workline.hr/CPortal/GeneralOpening.aspx?DetailCode=1</t>
         </is>
       </c>
-      <c r="C305" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C305" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D305" s="10" t="n"/>
@@ -12803,19 +12809,19 @@
       <c r="Z305" s="10" t="n"/>
     </row>
     <row r="306">
-      <c r="A306" s="52" t="inlineStr">
+      <c r="A306" s="43" t="inlineStr">
         <is>
           <t>BNY</t>
         </is>
       </c>
-      <c r="B306" s="53" t="inlineStr">
+      <c r="B306" s="44" t="inlineStr">
         <is>
           <t>https://bnymellon.eightfold.ai/careers?start=0&amp;location=India&amp;pid=40076775&amp;sort_by=distance&amp;filter_include_remote=1</t>
         </is>
       </c>
-      <c r="C306" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C306" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D306" s="10" t="n"/>
@@ -13043,19 +13049,19 @@
       <c r="Z311" s="10" t="n"/>
     </row>
     <row r="312">
-      <c r="A312" s="52" t="inlineStr">
+      <c r="A312" s="43" t="inlineStr">
         <is>
           <t>CBRE Group</t>
         </is>
       </c>
-      <c r="B312" s="53" t="inlineStr">
+      <c r="B312" s="44" t="inlineStr">
         <is>
           <t>https://careers.cbre.com/en_US/careers/SearchJobs/?9577=%5B17142%5D&amp;9577_format=10224&amp;listFilterMode=1&amp;jobSort=relevancy&amp;jobRecordsPerPage=25&amp;</t>
         </is>
       </c>
-      <c r="C312" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C312" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D312" s="10" t="n"/>
@@ -13123,20 +13129,20 @@
       <c r="Z313" s="10" t="n"/>
     </row>
     <row r="314">
-      <c r="A314" s="52" t="inlineStr">
+      <c r="A314" s="43" t="inlineStr">
         <is>
           <t>Cloudflare</t>
         </is>
       </c>
-      <c r="B314" s="58" t="inlineStr">
+      <c r="B314" s="45" t="inlineStr">
         <is>
           <t>https://www.cloudflare.com/en-in/careers/jobs/?location=Bengaluru%2C+India
 https://www.cloudflare.com/en-in/careers/jobs/?location=India</t>
         </is>
       </c>
-      <c r="C314" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C314" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D314" s="10" t="n"/>
@@ -13285,19 +13291,19 @@
       <c r="Z317" s="10" t="n"/>
     </row>
     <row r="318">
-      <c r="A318" s="52" t="inlineStr">
+      <c r="A318" s="43" t="inlineStr">
         <is>
           <t>Deutsche Bahn</t>
         </is>
       </c>
-      <c r="B318" s="53" t="inlineStr">
+      <c r="B318" s="44" t="inlineStr">
         <is>
           <t>https://db.jobs/service/search/en-en/5379744?query=International%20Jobs%20DB%20E.C.O.%20Group%20Deutsche%20bahn%20international%20operations%20gmbh&amp;location_awe=&amp;qli=true&amp;sort=pubExternalDate_tdt</t>
         </is>
       </c>
-      <c r="C318" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C318" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D318" s="10" t="n"/>
@@ -13325,19 +13331,19 @@
       <c r="Z318" s="10" t="n"/>
     </row>
     <row r="319">
-      <c r="A319" s="52" t="inlineStr">
+      <c r="A319" s="43" t="inlineStr">
         <is>
           <t>Deutsche Telekom</t>
         </is>
       </c>
-      <c r="B319" s="53" t="inlineStr">
+      <c r="B319" s="44" t="inlineStr">
         <is>
           <t>https://careers.telekom.com/en/jobs?location=India</t>
         </is>
       </c>
-      <c r="C319" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C319" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D319" s="10" t="n"/>
@@ -13405,19 +13411,19 @@
       <c r="Z320" s="10" t="n"/>
     </row>
     <row r="321">
-      <c r="A321" s="52" t="inlineStr">
+      <c r="A321" s="43" t="inlineStr">
         <is>
           <t>EaseMyTrip</t>
         </is>
       </c>
-      <c r="B321" s="53" t="inlineStr">
+      <c r="B321" s="44" t="inlineStr">
         <is>
           <t>https://www.easemytrip.com/career.html#work</t>
         </is>
       </c>
-      <c r="C321" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C321" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D321" s="10" t="n"/>
@@ -13485,20 +13491,20 @@
       <c r="Z322" s="10" t="n"/>
     </row>
     <row r="323">
-      <c r="A323" s="52" t="inlineStr">
+      <c r="A323" s="48" t="inlineStr">
         <is>
           <t>Eicher Motors</t>
         </is>
       </c>
-      <c r="B323" s="58" t="inlineStr">
+      <c r="B323" s="70" t="inlineStr">
         <is>
           <t>https://careers.vecv.in/search/?createNewAlert=false&amp;q=&amp;locationsearch=&amp;optionsFacetsDD_location=&amp;optionsFacetsDD_city=&amp;optionsFacetsDD_department=
 https://careers.royalenfield.com/us/en/home?_gl=1*y9ntof*_gcl_au*MjEyNTMxOTY3NC4xNzcxNTc2ODg5*_ga*MTUyNjI5NjQ3MC4xNzcxNTc2ODg5*_ga_7746PERT32*czE3NzE1NzY4ODkkbzEkZzEkdDE3NzE1NzY5MjAkajI5JGwwJGgw</t>
         </is>
       </c>
-      <c r="C323" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C323" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
         </is>
       </c>
       <c r="D323" s="10" t="n"/>
@@ -13526,19 +13532,19 @@
       <c r="Z323" s="10" t="n"/>
     </row>
     <row r="324">
-      <c r="A324" s="52" t="inlineStr">
+      <c r="A324" s="43" t="inlineStr">
         <is>
           <t>Electronic Arts</t>
         </is>
       </c>
-      <c r="B324" s="53" t="inlineStr">
+      <c r="B324" s="44" t="inlineStr">
         <is>
           <t>https://jobs.ea.com/en_US/careers/Home/?8171=%5B10590%5D&amp;8171_format=5683&amp;listFilterMode=1&amp;jobRecordsPerPage=20&amp;</t>
         </is>
       </c>
-      <c r="C324" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C324" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D324" s="10" t="n"/>
@@ -13566,19 +13572,19 @@
       <c r="Z324" s="10" t="n"/>
     </row>
     <row r="325">
-      <c r="A325" s="52" t="inlineStr">
+      <c r="A325" s="43" t="inlineStr">
         <is>
           <t>EPAM Systems</t>
         </is>
       </c>
-      <c r="B325" s="53" t="inlineStr">
+      <c r="B325" s="44" t="inlineStr">
         <is>
           <t>https://careers.epam.com/en/jobs?country=4060741400035606931</t>
         </is>
       </c>
-      <c r="C325" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C325" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D325" s="10" t="n"/>
@@ -13766,19 +13772,19 @@
       <c r="Z329" s="10" t="n"/>
     </row>
     <row r="330">
-      <c r="A330" s="52" t="inlineStr">
+      <c r="A330" s="43" t="inlineStr">
         <is>
           <t>Gallagher</t>
         </is>
       </c>
-      <c r="B330" s="53" t="inlineStr">
+      <c r="B330" s="44" t="inlineStr">
         <is>
           <t>https://jobs.ajg.com/ajg-global/jobs?locations=Bangalore,Karnataka,India%7CChandigarh,Punjab,India%7CGurugram,Haryana,India%7CMumbai,Maharashtra,India%7CPune,Maharashtra,India&amp;page=1</t>
         </is>
       </c>
-      <c r="C330" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C330" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D330" s="10" t="n"/>
@@ -13926,19 +13932,19 @@
       <c r="Z333" s="10" t="n"/>
     </row>
     <row r="334">
-      <c r="A334" s="52" t="inlineStr">
+      <c r="A334" s="43" t="inlineStr">
         <is>
           <t>Haptik</t>
         </is>
       </c>
-      <c r="B334" s="53" t="inlineStr">
+      <c r="B334" s="44" t="inlineStr">
         <is>
           <t>https://haptik.freshteam.com/jobs?__hstc=233858945.0eecb6901547789a76a8150b48139b47.1650872173205.1656650197197.1656654941825.85&amp;__hssc=233858945.2.1656654941825&amp;__hsfp=&amp;hsCtaTracking=be1d0f38-8578-466c-a65e-7dba125d958a%7C852c3dbe-26c9-4a01-a174-ad02a06686d9&amp;_gl=1*efxtfg*_gcl_au*Nzc1MDMyODQ4LjE3NzE1OTQwMTE.*_ga*ODU2MzA1MTQ2LjE3NzE1OTQwMTA.*_ga_TL7ZLD0W5B*czE3NzE1OTQwMDkkbzEkZzAkdDE3NzE1OTQwMDkkajYwJGwwJGgw</t>
         </is>
       </c>
-      <c r="C334" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C334" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D334" s="10" t="n"/>
@@ -13966,19 +13972,19 @@
       <c r="Z334" s="10" t="n"/>
     </row>
     <row r="335">
-      <c r="A335" s="52" t="inlineStr">
+      <c r="A335" s="43" t="inlineStr">
         <is>
           <t>Indegene</t>
         </is>
       </c>
-      <c r="B335" s="53" t="inlineStr">
+      <c r="B335" s="44" t="inlineStr">
         <is>
           <t>https://careers.indegene.com/search/?q=&amp;q2=&amp;alertId=&amp;locationsearch=&amp;facility=&amp;title=&amp;location=IN#searchresults</t>
         </is>
       </c>
-      <c r="C335" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C335" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D335" s="10" t="n"/>
@@ -14006,19 +14012,19 @@
       <c r="Z335" s="10" t="n"/>
     </row>
     <row r="336">
-      <c r="A336" s="52" t="inlineStr">
+      <c r="A336" s="43" t="inlineStr">
         <is>
           <t>Ingersoll Rand</t>
         </is>
       </c>
-      <c r="B336" s="53" t="inlineStr">
+      <c r="B336" s="44" t="inlineStr">
         <is>
           <t>https://careers.irco.com/go/Middle-East%2C-India-and-Africa/9515600/?q=&amp;q2=&amp;alertId=&amp;title=&amp;department=&amp;location=IN#searchresults</t>
         </is>
       </c>
-      <c r="C336" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C336" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D336" s="10" t="n"/>
@@ -14086,19 +14092,19 @@
       <c r="Z337" s="10" t="n"/>
     </row>
     <row r="338">
-      <c r="A338" s="52" t="inlineStr">
+      <c r="A338" s="43" t="inlineStr">
         <is>
           <t>Innovaccer</t>
         </is>
       </c>
-      <c r="B338" s="53" t="inlineStr">
+      <c r="B338" s="44" t="inlineStr">
         <is>
           <t>https://innovaccer.com/careers/jobs#view-jobs</t>
         </is>
       </c>
-      <c r="C338" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C338" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D338" s="10" t="n"/>

</xml_diff>

<commit_message>
feat: Add 49 new scrapers (Batches 19-20) for Fujitsu, Grant Thornton, Bloomberg, Canon, and more
Batch 19 (25 scrapers): WeWork, RPG Group, Axtria, Cargill, Odoo, Adidas, Ametek, UltraTech Cement,
Synopsys, Zee Entertainment, Amdocs, Cvent, Zebra Technologies, McDonald's, Quest Diagnostics,
Ralph Lauren, Zeiss, 7-Eleven, Welspun, Fynd, Societe Generale, WTW, NPCI, Rippling, Tata Technologies.

Batch 20 (24 scrapers): Ferrero, Essilor, Carlsberg, Seagate, Grab, Agility, Bloomberg, Skyscanner,
Gigamon, Boston Analytics, British Airways, Encore Capital, Zerodha, Shopify, TCIL, Fujitsu, Generali,
Four Seasons, ESPN, Gigabyte, Grant Thornton, Canon, Elevate, Vedantu.

33 working scrapers (758 total jobs), 21 broken. Notable: Fujitsu (150 jobs via SF API),
Grant Thornton (132 jobs via NaCl-encrypted TalentRecruit API). Total scrapers: 568.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company-list.xlsx
+++ b/company-list.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -81,6 +81,10 @@
     <font>
       <b val="1"/>
       <color rgb="009C6500"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="13">
@@ -169,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -364,6 +368,16 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -682,7 +696,7 @@
       <c r="A2" s="3" t="n"/>
       <c r="B2" s="27" t="inlineStr">
         <is>
-          <t>Done (544)</t>
+          <t>Done (583)</t>
         </is>
       </c>
       <c r="C2" s="10" t="n"/>
@@ -714,7 +728,7 @@
       <c r="A3" s="4" t="n"/>
       <c r="B3" s="28" t="inlineStr">
         <is>
-          <t>Pending (322)</t>
+          <t>Pending (267)</t>
         </is>
       </c>
       <c r="C3" s="10" t="n"/>
@@ -746,7 +760,7 @@
       <c r="A4" s="5" t="n"/>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>Broken (5)</t>
+          <t>Broken (21)</t>
         </is>
       </c>
       <c r="C4" s="10" t="n"/>
@@ -822,7 +836,11 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n"/>
+      <c r="D6" s="72" t="inlineStr">
+        <is>
+          <t>Job Count</t>
+        </is>
+      </c>
       <c r="E6" s="10" t="n"/>
       <c r="F6" s="10" t="n"/>
       <c r="G6" s="10" t="n"/>
@@ -10769,19 +10787,19 @@
       <c r="Z254" s="10" t="n"/>
     </row>
     <row r="255">
-      <c r="A255" s="52" t="inlineStr">
+      <c r="A255" s="43" t="inlineStr">
         <is>
           <t>Guangzhou Automobile Group</t>
         </is>
       </c>
-      <c r="B255" s="53" t="inlineStr">
+      <c r="B255" s="44" t="inlineStr">
         <is>
           <t>https://career.gac.com/?jobs-54d01ed5%5Bcountry%5D%5B%5D=IN</t>
         </is>
       </c>
-      <c r="C255" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C255" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D255" s="10" t="n"/>
@@ -12969,19 +12987,19 @@
       <c r="Z309" s="10" t="n"/>
     </row>
     <row r="310">
-      <c r="A310" s="52" t="inlineStr">
+      <c r="A310" s="43" t="inlineStr">
         <is>
           <t>CARS24</t>
         </is>
       </c>
-      <c r="B310" s="53" t="inlineStr">
+      <c r="B310" s="44" t="inlineStr">
         <is>
           <t>https://careers.cars24.com/</t>
         </is>
       </c>
-      <c r="C310" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C310" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D310" s="10" t="n"/>
@@ -14532,19 +14550,19 @@
       <c r="Z348" s="10" t="n"/>
     </row>
     <row r="349">
-      <c r="A349" s="52" t="inlineStr">
+      <c r="A349" s="43" t="inlineStr">
         <is>
           <t>Max Group</t>
         </is>
       </c>
-      <c r="B349" s="53" t="inlineStr">
+      <c r="B349" s="44" t="inlineStr">
         <is>
           <t>https://careers.maxlifeinsurance.com/search/?createNewAlert=false&amp;q=&amp;locationsearch=&amp;optionsFacetsDD_location=&amp;optionsFacetsDD_country=&amp;optionsFacetsDD_state=&amp;optionsFacetsDD_city=</t>
         </is>
       </c>
-      <c r="C349" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C349" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D349" s="10" t="n"/>
@@ -14572,22 +14590,24 @@
       <c r="Z349" s="10" t="n"/>
     </row>
     <row r="350">
-      <c r="A350" s="52" t="inlineStr">
+      <c r="A350" s="43" t="inlineStr">
         <is>
           <t>McDonald's</t>
         </is>
       </c>
-      <c r="B350" s="53" t="inlineStr">
+      <c r="B350" s="44" t="inlineStr">
         <is>
           <t>https://talent500.com/jobs/mcdonaldsindia/</t>
         </is>
       </c>
-      <c r="C350" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D350" s="10" t="n"/>
+      <c r="C350" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D350" s="43" t="n">
+        <v>20</v>
+      </c>
       <c r="E350" s="10" t="n"/>
       <c r="F350" s="10" t="n"/>
       <c r="G350" s="10" t="n"/>
@@ -14652,19 +14672,19 @@
       <c r="Z351" s="10" t="n"/>
     </row>
     <row r="352">
-      <c r="A352" s="52" t="inlineStr">
+      <c r="A352" s="48" t="inlineStr">
         <is>
           <t>National Payments Corporation of India</t>
         </is>
       </c>
-      <c r="B352" s="53" t="inlineStr">
+      <c r="B352" s="49" t="inlineStr">
         <is>
           <t>https://www.npci.org.in/careers</t>
         </is>
       </c>
-      <c r="C352" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C352" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
         </is>
       </c>
       <c r="D352" s="10" t="n"/>
@@ -14692,22 +14712,24 @@
       <c r="Z352" s="10" t="n"/>
     </row>
     <row r="353">
-      <c r="A353" s="52" t="inlineStr">
+      <c r="A353" s="43" t="inlineStr">
         <is>
           <t>Odoo</t>
         </is>
       </c>
-      <c r="B353" s="53" t="inlineStr">
+      <c r="B353" s="44" t="inlineStr">
         <is>
           <t>https://www.odoo.com/jobs</t>
         </is>
       </c>
-      <c r="C353" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D353" s="10" t="n"/>
+      <c r="C353" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D353" s="43" t="n">
+        <v>12</v>
+      </c>
       <c r="E353" s="10" t="n"/>
       <c r="F353" s="10" t="n"/>
       <c r="G353" s="10" t="n"/>
@@ -14972,22 +14994,24 @@
       <c r="Z359" s="10" t="n"/>
     </row>
     <row r="360">
-      <c r="A360" s="52" t="inlineStr">
+      <c r="A360" s="43" t="inlineStr">
         <is>
           <t>Quest Diagnostics</t>
         </is>
       </c>
-      <c r="B360" s="53" t="inlineStr">
+      <c r="B360" s="44" t="inlineStr">
         <is>
           <t>https://indiacareers.questdiagnostics.com/location/india-jobs/38852/1269750/2</t>
         </is>
       </c>
-      <c r="C360" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D360" s="10" t="n"/>
+      <c r="C360" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D360" s="43" t="n">
+        <v>4</v>
+      </c>
       <c r="E360" s="10" t="n"/>
       <c r="F360" s="10" t="n"/>
       <c r="G360" s="10" t="n"/>
@@ -15012,22 +15036,24 @@
       <c r="Z360" s="10" t="n"/>
     </row>
     <row r="361">
-      <c r="A361" s="52" t="inlineStr">
+      <c r="A361" s="43" t="inlineStr">
         <is>
           <t>Ralph Lauren Corporation</t>
         </is>
       </c>
-      <c r="B361" s="53" t="inlineStr">
+      <c r="B361" s="44" t="inlineStr">
         <is>
           <t>https://careers.ralphlauren.com/CareersCorporate/SearchJobsCorporate/?3413=3312571&amp;3413_format=1848&amp;listFilterMode=1</t>
         </is>
       </c>
-      <c r="C361" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D361" s="10" t="n"/>
+      <c r="C361" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D361" s="43" t="n">
+        <v>20</v>
+      </c>
       <c r="E361" s="10" t="n"/>
       <c r="F361" s="10" t="n"/>
       <c r="G361" s="10" t="n"/>
@@ -15052,19 +15078,19 @@
       <c r="Z361" s="10" t="n"/>
     </row>
     <row r="362">
-      <c r="A362" s="52" t="inlineStr">
+      <c r="A362" s="48" t="inlineStr">
         <is>
           <t>Rippling</t>
         </is>
       </c>
-      <c r="B362" s="53" t="inlineStr">
+      <c r="B362" s="49" t="inlineStr">
         <is>
           <t>https://www.rippling.com/en-GB/careers/open-roles</t>
         </is>
       </c>
-      <c r="C362" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C362" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
         </is>
       </c>
       <c r="D362" s="10" t="n"/>
@@ -15160,19 +15186,19 @@
       </c>
     </row>
     <row r="367">
-      <c r="A367" s="52" t="inlineStr">
+      <c r="A367" s="48" t="inlineStr">
         <is>
           <t>Fynd</t>
         </is>
       </c>
-      <c r="B367" s="53" t="inlineStr">
+      <c r="B367" s="49" t="inlineStr">
         <is>
           <t>https://www.fynd.com/careers#open-positions</t>
         </is>
       </c>
-      <c r="C367" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C367" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
         </is>
       </c>
     </row>
@@ -15187,28 +15213,34 @@
           <t>https://7-eleven-gsc.ripplehire.com/candidate/?token=AdexT4WYTKbaWH7lieeK&amp;lang=en&amp;source=LINKEDIN&amp;ref=LI02#list</t>
         </is>
       </c>
-      <c r="C368" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C368" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D368" s="0" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="369">
-      <c r="A369" s="52" t="inlineStr">
+      <c r="A369" s="43" t="inlineStr">
         <is>
           <t>UltraTech Cement</t>
         </is>
       </c>
-      <c r="B369" s="59" t="inlineStr">
+      <c r="B369" s="46" t="inlineStr">
         <is>
           <t>https://abgcareers.peoplestrong.com/job/joblist
 Org Unit: Cement</t>
         </is>
       </c>
-      <c r="C369" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C369" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D369" s="65" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="370">
@@ -15229,105 +15261,114 @@
       </c>
     </row>
     <row r="371">
-      <c r="A371" s="52" t="inlineStr">
+      <c r="A371" s="48" t="inlineStr">
         <is>
           <t>Société Générale</t>
         </is>
       </c>
-      <c r="B371" s="53" t="inlineStr">
+      <c r="B371" s="49" t="inlineStr">
         <is>
           <t>https://careers.societegenerale.com/en/search?refinementList[jobLocation][0]=IND</t>
         </is>
       </c>
-      <c r="C371" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C371" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
         </is>
       </c>
     </row>
     <row r="372">
-      <c r="A372" s="52" t="inlineStr">
+      <c r="A372" s="43" t="inlineStr">
         <is>
           <t>Synopsys</t>
         </is>
       </c>
-      <c r="B372" s="53" t="inlineStr">
+      <c r="B372" s="44" t="inlineStr">
         <is>
           <t>https://careers.synopsys.com/search-jobs</t>
         </is>
       </c>
-      <c r="C372" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C372" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D372" s="65" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="373">
-      <c r="A373" s="52" t="inlineStr">
+      <c r="A373" s="43" t="inlineStr">
         <is>
           <t>Urban Company</t>
         </is>
       </c>
-      <c r="B373" s="53" t="inlineStr">
+      <c r="B373" s="44" t="inlineStr">
         <is>
           <t>https://careers.urbancompany.com/jobs</t>
         </is>
       </c>
-      <c r="C373" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C373" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="374">
-      <c r="A374" s="52" t="inlineStr">
+      <c r="A374" s="48" t="inlineStr">
         <is>
           <t>Willis Towers Watson</t>
         </is>
       </c>
-      <c r="B374" s="53" t="inlineStr">
+      <c r="B374" s="49" t="inlineStr">
         <is>
           <t>https://careers.wtwco.com/jobs/search?page=1&amp;country_codes%5B%5D=IN&amp;query=</t>
         </is>
       </c>
-      <c r="C374" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C374" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
         </is>
       </c>
     </row>
     <row r="375">
-      <c r="A375" s="52" t="inlineStr">
+      <c r="A375" s="43" t="inlineStr">
         <is>
           <t>Zebra Technologies</t>
         </is>
       </c>
-      <c r="B375" s="53" t="inlineStr">
+      <c r="B375" s="44" t="inlineStr">
         <is>
           <t>https://careers.zebra.com/careers</t>
         </is>
       </c>
-      <c r="C375" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C375" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D375" s="65" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="376">
-      <c r="A376" s="52" t="inlineStr">
+      <c r="A376" s="43" t="inlineStr">
         <is>
           <t>RPG Group</t>
         </is>
       </c>
-      <c r="B376" s="53" t="inlineStr">
+      <c r="B376" s="44" t="inlineStr">
         <is>
           <t>https://jobs.rpggroup.com/search/?createNewAlert=false&amp;q=</t>
         </is>
       </c>
-      <c r="C376" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C376" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D376" s="65" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="377">
@@ -15348,36 +15389,36 @@
       </c>
     </row>
     <row r="378">
-      <c r="A378" s="52" t="inlineStr">
+      <c r="A378" s="43" t="inlineStr">
         <is>
           <t>ShareChat</t>
         </is>
       </c>
-      <c r="B378" s="53" t="inlineStr">
+      <c r="B378" s="44" t="inlineStr">
         <is>
           <t>https://sharechat.com/careers</t>
         </is>
       </c>
-      <c r="C378" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C378" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="379">
-      <c r="A379" s="52" t="inlineStr">
+      <c r="A379" s="48" t="inlineStr">
         <is>
           <t>Tata Technologies</t>
         </is>
       </c>
-      <c r="B379" s="53" t="inlineStr">
+      <c r="B379" s="49" t="inlineStr">
         <is>
           <t>https://tatatechnologies.ripplehire.com/candidate/?token=pUMIYomQw46RCgLl0Cyq&amp;lang=en&amp;source=CAREERSITE#list/bu=INDIA</t>
         </is>
       </c>
-      <c r="C379" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C379" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
         </is>
       </c>
     </row>
@@ -15399,37 +15440,43 @@
       </c>
     </row>
     <row r="381">
-      <c r="A381" s="52" t="inlineStr">
+      <c r="A381" s="43" t="inlineStr">
         <is>
           <t>Welspun</t>
         </is>
       </c>
-      <c r="B381" s="53" t="inlineStr">
+      <c r="B381" s="44" t="inlineStr">
         <is>
           <t>https://welpro.welspun.com/careers?SiteName=jSIHd9FMCv/kd6koxIV5bVFzdqnRhv7lEcsAW5OEjUs=</t>
         </is>
       </c>
-      <c r="C381" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C381" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D381" s="65" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="382">
-      <c r="A382" s="52" t="inlineStr">
+      <c r="A382" s="43" t="inlineStr">
         <is>
           <t>WeWork</t>
         </is>
       </c>
-      <c r="B382" s="53" t="inlineStr">
+      <c r="B382" s="44" t="inlineStr">
         <is>
           <t>https://weworkindia.hire.trakstar.com/</t>
         </is>
       </c>
-      <c r="C382" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C382" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D382" s="65" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="383">
@@ -15467,20 +15514,23 @@
       </c>
     </row>
     <row r="385">
-      <c r="A385" s="52" t="inlineStr">
+      <c r="A385" s="43" t="inlineStr">
         <is>
           <t>Zee Entertainment Enterprises</t>
         </is>
       </c>
-      <c r="B385" s="53" t="inlineStr">
+      <c r="B385" s="44" t="inlineStr">
         <is>
           <t>https://zee.sensehq.com/careers</t>
         </is>
       </c>
-      <c r="C385" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C385" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D385" s="65" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="386">
@@ -15518,20 +15568,23 @@
       </c>
     </row>
     <row r="388">
-      <c r="A388" s="62" t="inlineStr">
+      <c r="A388" s="60" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="B388" s="63" t="inlineStr">
+      <c r="B388" s="61" t="inlineStr">
         <is>
           <t>https://careers.adidas-group.com/jobs?brand=&amp;team=&amp;type=&amp;keywords=&amp;location=%5B%7B%22country%22%3A%22India%22%7D%5D&amp;sort=&amp;locale=en&amp;offset=0</t>
         </is>
       </c>
-      <c r="C388" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C388" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D388" s="65" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="389">
@@ -15552,20 +15605,23 @@
       </c>
     </row>
     <row r="390">
-      <c r="A390" s="62" t="inlineStr">
+      <c r="A390" s="60" t="inlineStr">
         <is>
           <t>Amdocs</t>
         </is>
       </c>
-      <c r="B390" s="63" t="inlineStr">
+      <c r="B390" s="61" t="inlineStr">
         <is>
           <t>https://jobs.amdocs.com/careers?_gl=1*15dwam3*_gcl_au*MTYwNTkzMTc1OS4xNzcyMDE2OTU3*_ga*MTg3Nzg4OTE0LjE3NzIwMTY5NTY.*_ga_EVYPKWJHSE*czE3NzIwMTY5NTYkbzEkZzEkdDE3NzIwMTY5NTYkajYwJGwwJGgw&amp;start=0&amp;location=IN&amp;pid=563431012320217&amp;sort_by=distance&amp;filter_include_remote=1</t>
         </is>
       </c>
-      <c r="C390" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C390" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D390" s="65" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="391">
@@ -15586,20 +15642,23 @@
       </c>
     </row>
     <row r="392">
-      <c r="A392" s="62" t="inlineStr">
+      <c r="A392" s="60" t="inlineStr">
         <is>
           <t>Ametek</t>
         </is>
       </c>
-      <c r="B392" s="63" t="inlineStr">
+      <c r="B392" s="61" t="inlineStr">
         <is>
           <t>https://jobs.ametek.com/search/?q=&amp;q2=&amp;alertId=&amp;title=&amp;location=IN&amp;date=#searchresults</t>
         </is>
       </c>
-      <c r="C392" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C392" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D392" s="65" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="393">
@@ -15637,20 +15696,23 @@
       </c>
     </row>
     <row r="395">
-      <c r="A395" s="62" t="inlineStr">
+      <c r="A395" s="60" t="inlineStr">
         <is>
           <t>Axtria</t>
         </is>
       </c>
-      <c r="B395" s="63" t="inlineStr">
+      <c r="B395" s="61" t="inlineStr">
         <is>
           <t>https://www.axtria.com/axtria-careers/</t>
         </is>
       </c>
-      <c r="C395" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C395" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D395" s="65" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="396">
@@ -15671,37 +15733,43 @@
       </c>
     </row>
     <row r="397">
-      <c r="A397" s="62" t="inlineStr">
+      <c r="A397" s="60" t="inlineStr">
         <is>
           <t>Cargill</t>
         </is>
       </c>
-      <c r="B397" s="63" t="inlineStr">
+      <c r="B397" s="61" t="inlineStr">
         <is>
           <t>https://careers.cargill.com/en/search-jobs</t>
         </is>
       </c>
-      <c r="C397" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C397" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D397" s="65" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="398">
-      <c r="A398" s="62" t="inlineStr">
+      <c r="A398" s="60" t="inlineStr">
         <is>
           <t>Zeiss</t>
         </is>
       </c>
-      <c r="B398" s="63" t="inlineStr">
+      <c r="B398" s="61" t="inlineStr">
         <is>
           <t>https://www.zeiss.com/career/en/job-search.html?page=1&amp;locations=Ahmedabad%2C+India%2CBangalore%2C+India%2CChandigarh%2C+India%2CCoimbatore%2C+India%2CGurgaon%2C+India%2CHyderabad%2C+India%2CJaipur%2C+India%2CKolkata%2C+India%2CLucknow%2C+India%2CLudhiana%2C+India%2CMadurai%2C+India%2CNew+Delhi%2C+India%2CPune%2C+India%2CSurat%2C+India%2CVaranasi%2C+India%2Ccountry%3Aindia</t>
         </is>
       </c>
-      <c r="C398" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C398" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D398" s="65" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="399">
@@ -15739,37 +15807,43 @@
       </c>
     </row>
     <row r="401">
-      <c r="A401" s="62" t="inlineStr">
+      <c r="A401" s="60" t="inlineStr">
         <is>
           <t>Cvent</t>
         </is>
       </c>
-      <c r="B401" s="63" t="inlineStr">
+      <c r="B401" s="61" t="inlineStr">
         <is>
           <t>https://careers.cvent.com/jobs?limit=100&amp;page=1&amp;location=India&amp;stretch=10&amp;stretchUnit=MILES</t>
         </is>
       </c>
-      <c r="C401" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C401" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D401" s="65" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="402">
-      <c r="A402" s="62" t="inlineStr">
+      <c r="A402" s="60" t="inlineStr">
         <is>
           <t>Ferrero</t>
         </is>
       </c>
-      <c r="B402" s="63" t="inlineStr">
+      <c r="B402" s="61" t="inlineStr">
         <is>
           <t>https://www.ferrerocareers.com/int/en/jobs?search_country=Ind&amp;country[India]=India</t>
         </is>
       </c>
-      <c r="C402" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C402" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D402" s="65" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="403">
@@ -15790,20 +15864,23 @@
       </c>
     </row>
     <row r="404">
-      <c r="A404" s="62" t="inlineStr">
+      <c r="A404" s="60" t="inlineStr">
         <is>
           <t>Fujitsu</t>
         </is>
       </c>
-      <c r="B404" s="63" t="inlineStr">
+      <c r="B404" s="61" t="inlineStr">
         <is>
           <t>https://www.jobs.global.fujitsu.com/search/?q=&amp;locationsearch=&amp;searchResultView=LIST&amp;markerViewed=&amp;carouselIndex=&amp;facetFilters=%7B%22jobLocationCountry%22%3A%5B%22India%22%5D%7D&amp;pageNumber=0</t>
         </is>
       </c>
-      <c r="C404" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C404" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D404" s="65" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="405">
@@ -15841,20 +15918,23 @@
       </c>
     </row>
     <row r="407">
-      <c r="A407" s="62" t="inlineStr">
+      <c r="A407" s="60" t="inlineStr">
         <is>
           <t>Generali</t>
         </is>
       </c>
-      <c r="B407" s="63" t="inlineStr">
+      <c r="B407" s="61" t="inlineStr">
         <is>
           <t>https://www.generalicentralinsurance.com/current-openings</t>
         </is>
       </c>
-      <c r="C407" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C407" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D407" s="65" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="408">
@@ -15892,21 +15972,22 @@
       </c>
     </row>
     <row r="410">
-      <c r="A410" s="62" t="inlineStr">
+      <c r="A410" s="73" t="inlineStr">
         <is>
           <t>Grab Taxi</t>
         </is>
       </c>
-      <c r="B410" s="63" t="inlineStr">
+      <c r="B410" s="74" t="inlineStr">
         <is>
           <t>https://www.grab.careers/en/jobs/?search=&amp;country=India&amp;pagesize=20#results</t>
         </is>
       </c>
-      <c r="C410" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="C410" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D410" s="75" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="60" t="inlineStr">
@@ -15960,20 +16041,23 @@
       </c>
     </row>
     <row r="414">
-      <c r="A414" s="62" t="inlineStr">
+      <c r="A414" s="60" t="inlineStr">
         <is>
           <t>Four Seasons Hotels And Resorts</t>
         </is>
       </c>
-      <c r="B414" s="63" t="inlineStr">
+      <c r="B414" s="61" t="inlineStr">
         <is>
           <t>https://careers.fourseasons.com/us/en/search-results</t>
         </is>
       </c>
-      <c r="C414" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C414" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D414" s="65" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="415">
@@ -15994,37 +16078,41 @@
       </c>
     </row>
     <row r="416">
-      <c r="A416" s="62" t="inlineStr">
+      <c r="A416" s="73" t="inlineStr">
         <is>
           <t>ESPN</t>
         </is>
       </c>
-      <c r="B416" s="63" t="inlineStr">
+      <c r="B416" s="74" t="inlineStr">
         <is>
           <t>https://jobs.disneycareers.com/search-jobs?acm=ALL&amp;alrpm=ALL&amp;ascf=[%7B%22key%22:%22custom_fields.IndustryCustomField%22,%22value%22:%22ESPN%22%7D]</t>
         </is>
       </c>
-      <c r="C416" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="C416" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D416" s="75" t="n"/>
     </row>
     <row r="417">
-      <c r="A417" s="62" t="inlineStr">
+      <c r="A417" s="60" t="inlineStr">
         <is>
           <t>Essilor</t>
         </is>
       </c>
-      <c r="B417" s="63" t="inlineStr">
+      <c r="B417" s="61" t="inlineStr">
         <is>
           <t>https://careers.essilorluxottica.com/search/?createNewAlert=false&amp;q=&amp;optionsFacetsDD_country=IN&amp;optionsFacetsDD_city=&amp;optionsFacetsDD_customfield1=&amp;optionsFacetsDD_customfield2=&amp;optionsFacetsDD_customfield3=&amp;optionsFacetsDD_customfield4=</t>
         </is>
       </c>
-      <c r="C417" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C417" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D417" s="65" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="418">
@@ -16045,72 +16133,78 @@
       </c>
     </row>
     <row r="419">
-      <c r="A419" s="62" t="inlineStr">
+      <c r="A419" s="73" t="inlineStr">
         <is>
           <t>Gigabyte</t>
         </is>
       </c>
-      <c r="B419" s="63" t="inlineStr">
+      <c r="B419" s="74" t="inlineStr">
         <is>
           <t>https://www.gigabyte.com/in/Career/-6</t>
         </is>
       </c>
-      <c r="C419" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="C419" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D419" s="75" t="n"/>
     </row>
     <row r="420">
-      <c r="A420" s="62" t="inlineStr">
+      <c r="A420" s="73" t="inlineStr">
         <is>
           <t>Gigamon</t>
         </is>
       </c>
-      <c r="B420" s="63" t="inlineStr">
+      <c r="B420" s="74" t="inlineStr">
         <is>
           <t>https://jobs.jobvite.com/gigamon/search?intcid=careers-india</t>
         </is>
       </c>
-      <c r="C420" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="C420" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D420" s="75" t="n"/>
     </row>
     <row r="421">
-      <c r="A421" s="62" t="inlineStr">
+      <c r="A421" s="60" t="inlineStr">
         <is>
           <t>Grant Thornton</t>
         </is>
       </c>
-      <c r="B421" s="63" t="inlineStr">
+      <c r="B421" s="61" t="inlineStr">
         <is>
           <t>https://gtprod.talentrecruit.com/career-page</t>
         </is>
       </c>
-      <c r="C421" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C421" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D421" s="65" t="n">
+        <v>132</v>
       </c>
     </row>
     <row r="422">
-      <c r="A422" s="62" t="inlineStr">
+      <c r="A422" s="73" t="inlineStr">
         <is>
           <t>Agility</t>
         </is>
       </c>
-      <c r="B422" s="63" t="inlineStr">
+      <c r="B422" s="74" t="inlineStr">
         <is>
           <t>https://apply.workable.com/agility/</t>
         </is>
       </c>
-      <c r="C422" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="C422" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D422" s="75" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="62" t="inlineStr">
@@ -16140,10 +16234,13 @@
           <t>https://careers.zebra.com/careers?location=India&amp;pid=343636467416&amp;domain=zebra.com&amp;sort_by=relevance&amp;triggerGoButton=true&amp;triggerGoButton=false</t>
         </is>
       </c>
-      <c r="C424" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C424" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D424" s="0" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="425">
@@ -16198,122 +16295,141 @@
       </c>
     </row>
     <row r="428">
-      <c r="A428" s="62" t="inlineStr">
+      <c r="A428" s="60" t="inlineStr">
         <is>
           <t>Bloomberg</t>
         </is>
       </c>
-      <c r="B428" s="63" t="inlineStr">
+      <c r="B428" s="61" t="inlineStr">
         <is>
           <t>https://bloomberg.avature.net/careers/SearchJobs/?1845=%5B162477%2C162478%2C162575%5D&amp;1845_format=3996&amp;listFilterMode=1&amp;jobRecordsPerPage=12&amp;</t>
         </is>
       </c>
-      <c r="C428" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C428" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D428" s="65" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="429">
-      <c r="A429" s="62" t="inlineStr">
+      <c r="A429" s="60" t="inlineStr">
         <is>
           <t>Boston Analytics</t>
         </is>
       </c>
-      <c r="B429" s="63" t="inlineStr">
+      <c r="B429" s="61" t="inlineStr">
         <is>
           <t>https://bostonanalytics.com/careers.php</t>
         </is>
       </c>
-      <c r="C429" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C429" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D429" s="65" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="430">
-      <c r="A430" s="62" t="inlineStr">
+      <c r="A430" s="73" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="B430" s="63" t="inlineStr">
+      <c r="B430" s="74" t="inlineStr">
         <is>
           <t>https://careers.ba.com/search-jobs</t>
         </is>
       </c>
-      <c r="C430" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="C430" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D430" s="75" t="n"/>
     </row>
     <row r="431">
-      <c r="A431" s="62" t="inlineStr">
+      <c r="A431" s="60" t="inlineStr">
         <is>
           <t>Canon</t>
         </is>
       </c>
-      <c r="B431" s="63" t="inlineStr">
+      <c r="B431" s="61" t="inlineStr">
         <is>
           <t>https://career.asia.canon:8086/psc/ps/EMPLOYEE/CIPLCAREER/c/HRS_HRAM.HRS_APP_SCHJOB.GBL?Page=HRS_APP_SCHJOB&amp;Action=U&amp;FOCUS=Applicant&amp;SiteId=2226&amp;</t>
         </is>
       </c>
-      <c r="C431" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C431" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D431" s="65" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="432">
-      <c r="A432" s="62" t="inlineStr">
+      <c r="A432" s="60" t="inlineStr">
         <is>
           <t>Carlsberg Group</t>
         </is>
       </c>
-      <c r="B432" s="63" t="inlineStr">
+      <c r="B432" s="61" t="inlineStr">
         <is>
           <t>https://careers.carlsberg.com/search/?createNewAlert=false&amp;q=&amp;locationsearch=IN&amp;optionsFacetsDD_customfield1=&amp;optionsFacetsDD_customfield3=&amp;optionsFacetsDD_customfield2=</t>
         </is>
       </c>
-      <c r="C432" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C432" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D432" s="65" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="433">
-      <c r="A433" s="62" t="inlineStr">
+      <c r="A433" s="60" t="inlineStr">
         <is>
           <t>Elevate</t>
         </is>
       </c>
-      <c r="B433" s="63" t="inlineStr">
+      <c r="B433" s="61" t="inlineStr">
         <is>
           <t>https://elevate.law/explore-elevate-global/#opportunities</t>
         </is>
       </c>
-      <c r="C433" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C433" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D433" s="65" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="434">
-      <c r="A434" s="62" t="inlineStr">
+      <c r="A434" s="60" t="inlineStr">
         <is>
           <t>Encore Capital Group</t>
         </is>
       </c>
-      <c r="B434" s="63" t="inlineStr">
+      <c r="B434" s="61" t="inlineStr">
         <is>
           <t>https://careers.encorecapital.com/en/search-jobs</t>
         </is>
       </c>
-      <c r="C434" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+      <c r="C434" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D434" s="65" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="435">
@@ -16397,22 +16513,22 @@
       <c r="Z436" s="10" t="n"/>
     </row>
     <row r="437">
-      <c r="A437" s="52" t="inlineStr">
+      <c r="A437" s="48" t="inlineStr">
         <is>
           <t>Zerodha</t>
         </is>
       </c>
-      <c r="B437" s="53" t="inlineStr">
+      <c r="B437" s="49" t="inlineStr">
         <is>
           <t>https://careers.zerodha.com/</t>
         </is>
       </c>
-      <c r="C437" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D437" s="10" t="n"/>
+      <c r="C437" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D437" s="48" t="n"/>
       <c r="E437" s="10" t="n"/>
       <c r="F437" s="10" t="n"/>
       <c r="G437" s="10" t="n"/>
@@ -16557,22 +16673,24 @@
       <c r="Z440" s="10" t="n"/>
     </row>
     <row r="441">
-      <c r="A441" s="52" t="inlineStr">
+      <c r="A441" s="43" t="inlineStr">
         <is>
           <t>Seagate Technology</t>
         </is>
       </c>
-      <c r="B441" s="53" t="inlineStr">
+      <c r="B441" s="44" t="inlineStr">
         <is>
           <t>https://seagatecareers.com/search/?createNewAlert=false&amp;q=&amp;locationsearch=IN&amp;optionsFacetsDD_country=&amp;optionsFacetsDD_dept=&amp;optionsFacetsDD_customfield1=&amp;optionsFacetsDD_lang=</t>
         </is>
       </c>
-      <c r="C441" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D441" s="10" t="n"/>
+      <c r="C441" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D441" s="43" t="n">
+        <v>2</v>
+      </c>
       <c r="E441" s="10" t="n"/>
       <c r="F441" s="10" t="n"/>
       <c r="G441" s="10" t="n"/>
@@ -16597,22 +16715,22 @@
       <c r="Z441" s="10" t="n"/>
     </row>
     <row r="442">
-      <c r="A442" s="52" t="inlineStr">
+      <c r="A442" s="48" t="inlineStr">
         <is>
           <t>Transport Corporation of India</t>
         </is>
       </c>
-      <c r="B442" s="53" t="inlineStr">
+      <c r="B442" s="49" t="inlineStr">
         <is>
           <t>https://tcil.com/careers/</t>
         </is>
       </c>
-      <c r="C442" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D442" s="10" t="n"/>
+      <c r="C442" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D442" s="48" t="n"/>
       <c r="E442" s="10" t="n"/>
       <c r="F442" s="10" t="n"/>
       <c r="G442" s="10" t="n"/>
@@ -16637,22 +16755,24 @@
       <c r="Z442" s="10" t="n"/>
     </row>
     <row r="443">
-      <c r="A443" s="52" t="inlineStr">
+      <c r="A443" s="43" t="inlineStr">
         <is>
           <t>Vedantu</t>
         </is>
       </c>
-      <c r="B443" s="53" t="inlineStr">
+      <c r="B443" s="44" t="inlineStr">
         <is>
           <t>https://vedantu.zohorecruit.in/jobs/Careers</t>
         </is>
       </c>
-      <c r="C443" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D443" s="10" t="n"/>
+      <c r="C443" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D443" s="43" t="n">
+        <v>2</v>
+      </c>
       <c r="E443" s="10" t="n"/>
       <c r="F443" s="10" t="n"/>
       <c r="G443" s="10" t="n"/>
@@ -16797,22 +16917,22 @@
       <c r="Z446" s="10" t="n"/>
     </row>
     <row r="447">
-      <c r="A447" s="52" t="inlineStr">
+      <c r="A447" s="48" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="B447" s="53" t="inlineStr">
+      <c r="B447" s="49" t="inlineStr">
         <is>
           <t>https://www.shopify.com/careers?keyword=India#WhatWeDo</t>
         </is>
       </c>
-      <c r="C447" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D447" s="10" t="n"/>
+      <c r="C447" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D447" s="48" t="n"/>
       <c r="E447" s="10" t="n"/>
       <c r="F447" s="10" t="n"/>
       <c r="G447" s="10" t="n"/>
@@ -16837,22 +16957,22 @@
       <c r="Z447" s="10" t="n"/>
     </row>
     <row r="448">
-      <c r="A448" s="52" t="inlineStr">
+      <c r="A448" s="48" t="inlineStr">
         <is>
           <t>Skyscanner</t>
         </is>
       </c>
-      <c r="B448" s="53" t="inlineStr">
+      <c r="B448" s="49" t="inlineStr">
         <is>
           <t>https://www.skyscanner.co.in/jobs/current-jobs</t>
         </is>
       </c>
-      <c r="C448" s="34" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D448" s="10" t="n"/>
+      <c r="C448" s="71" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="D448" s="48" t="n"/>
       <c r="E448" s="10" t="n"/>
       <c r="F448" s="10" t="n"/>
       <c r="G448" s="10" t="n"/>

</xml_diff>